<commit_message>
updated to si-6 0.20.32
</commit_message>
<xml_diff>
--- a/auto_repair/public/www/assets/xlsx/si-6.xlsx
+++ b/auto_repair/public/www/assets/xlsx/si-6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abees\Documents\sic\auto-repair-erp\web\src\assets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15BFA07-2AFD-45E6-BDDD-2C1A998743FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656B2AB4-843D-46E1-91CF-15469E79002C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fiscal Years" sheetId="1" r:id="rId1"/>
@@ -32,9 +32,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Journal Entries'!$A$1:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Products!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Raw Material'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Trading!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Products!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Raw Material'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Trading!$A$1:$H$1</definedName>
     <definedName name="arial" localSheetId="13">Invoices!$1:$1048576</definedName>
     <definedName name="arial">#REF!</definedName>
   </definedNames>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="125">
   <si>
     <t>year</t>
   </si>
@@ -429,6 +429,9 @@
   </si>
   <si>
     <t>system</t>
+  </si>
+  <si>
+    <t>Is Recycable</t>
   </si>
 </sst>
 </file>
@@ -1723,22 +1726,23 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD83FC68-3866-4B53-B82D-AC812A1EEF62}">
-  <dimension ref="A1:XFA1"/>
+  <dimension ref="A1:XFB1"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="13" customWidth="1"/>
     <col min="2" max="2" width="24.33203125" style="20" customWidth="1"/>
     <col min="3" max="3" width="36.88671875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" style="13" customWidth="1"/>
-    <col min="6" max="6" width="24.6640625" style="13" customWidth="1"/>
-    <col min="7" max="7" width="17" style="13" customWidth="1"/>
-    <col min="8" max="8" width="21.33203125" style="21" customWidth="1"/>
-    <col min="9" max="16381" width="11.5546875" style="13"/>
-    <col min="16382" max="16384" width="11.5546875" style="14"/>
+    <col min="4" max="4" width="17.6640625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="24.6640625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="17" style="13" customWidth="1"/>
+    <col min="9" max="9" width="21.33203125" style="21" customWidth="1"/>
+    <col min="10" max="16382" width="11.5546875" style="13"/>
+    <col min="16383" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="15" t="s">
         <v>116</v>
       </c>
@@ -1749,18 +1753,21 @@
         <v>106</v>
       </c>
       <c r="D1" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="H1" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="I1" s="21" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1777,22 +1784,23 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE5D49AE-AF0F-4668-A81E-764A0CB4B708}">
-  <dimension ref="A1:XFA1"/>
+  <dimension ref="A1:XFB1"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="28.109375" style="13" customWidth="1"/>
     <col min="2" max="2" width="24.33203125" style="20" customWidth="1"/>
     <col min="3" max="3" width="36.88671875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" style="13" customWidth="1"/>
-    <col min="6" max="6" width="24.6640625" style="13" customWidth="1"/>
-    <col min="7" max="7" width="17" style="13" customWidth="1"/>
-    <col min="8" max="8" width="21.6640625" style="21" customWidth="1"/>
-    <col min="9" max="16381" width="11.5546875" style="13"/>
-    <col min="16382" max="16384" width="11.5546875" style="14"/>
+    <col min="4" max="4" width="15.33203125" style="13" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="24.6640625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="17" style="13" customWidth="1"/>
+    <col min="9" max="9" width="21.6640625" style="21" customWidth="1"/>
+    <col min="10" max="16382" width="11.5546875" style="13"/>
+    <col min="16383" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="15" t="s">
         <v>116</v>
       </c>
@@ -1803,18 +1811,21 @@
         <v>106</v>
       </c>
       <c r="D1" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="H1" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="I1" s="21" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1830,23 +1841,23 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:XFB6"/>
+  <dimension ref="A1:XFC6"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="13" customWidth="1"/>
     <col min="2" max="2" width="16.88671875" style="20" customWidth="1"/>
-    <col min="3" max="3" width="18.88671875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="17.33203125" style="13" customWidth="1"/>
-    <col min="7" max="7" width="20.6640625" style="21" customWidth="1"/>
-    <col min="8" max="8" width="22.44140625" style="13" customWidth="1"/>
-    <col min="9" max="9" width="24" style="13" customWidth="1"/>
-    <col min="10" max="11" width="22.33203125" style="13" customWidth="1"/>
-    <col min="13" max="16382" width="11.5546875" style="13"/>
-    <col min="16383" max="16384" width="11.5546875" style="14"/>
+    <col min="3" max="4" width="18.88671875" style="13" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.33203125" style="13" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" style="21" customWidth="1"/>
+    <col min="9" max="9" width="22.44140625" style="13" customWidth="1"/>
+    <col min="10" max="10" width="24" style="13" customWidth="1"/>
+    <col min="11" max="12" width="22.33203125" style="13" customWidth="1"/>
+    <col min="14" max="16383" width="11.5546875" style="13"/>
+    <col min="16384" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="15" t="s">
         <v>116</v>
       </c>
@@ -1857,39 +1868,43 @@
         <v>106</v>
       </c>
       <c r="D1" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="H1" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="I1" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" s="15"/>
       <c r="B6" s="19"/>
       <c r="C6" s="15"/>
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="G6" s="15"/>
       <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>

</xml_diff>

<commit_message>
revert back to v0.20.30 for si-6 for nginx error
</commit_message>
<xml_diff>
--- a/auto_repair/public/www/assets/xlsx/si-6.xlsx
+++ b/auto_repair/public/www/assets/xlsx/si-6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abees\Documents\sic\auto-repair-erp\web\src\assets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656B2AB4-843D-46E1-91CF-15469E79002C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15BFA07-2AFD-45E6-BDDD-2C1A998743FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fiscal Years" sheetId="1" r:id="rId1"/>
@@ -32,9 +32,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Journal Entries'!$A$1:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Products!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Raw Material'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Trading!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Products!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Raw Material'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Trading!$A$1:$G$1</definedName>
     <definedName name="arial" localSheetId="13">Invoices!$1:$1048576</definedName>
     <definedName name="arial">#REF!</definedName>
   </definedNames>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="124">
   <si>
     <t>year</t>
   </si>
@@ -429,9 +429,6 @@
   </si>
   <si>
     <t>system</t>
-  </si>
-  <si>
-    <t>Is Recycable</t>
   </si>
 </sst>
 </file>
@@ -1726,23 +1723,22 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD83FC68-3866-4B53-B82D-AC812A1EEF62}">
-  <dimension ref="A1:XFB1"/>
+  <dimension ref="A1:XFA1"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="13" customWidth="1"/>
     <col min="2" max="2" width="24.33203125" style="20" customWidth="1"/>
     <col min="3" max="3" width="36.88671875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" style="13" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" style="13" customWidth="1"/>
-    <col min="7" max="7" width="24.6640625" style="13" customWidth="1"/>
-    <col min="8" max="8" width="17" style="13" customWidth="1"/>
-    <col min="9" max="9" width="21.33203125" style="21" customWidth="1"/>
-    <col min="10" max="16382" width="11.5546875" style="13"/>
-    <col min="16383" max="16384" width="11.5546875" style="14"/>
+    <col min="4" max="4" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" style="13" customWidth="1"/>
+    <col min="6" max="6" width="24.6640625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="17" style="13" customWidth="1"/>
+    <col min="8" max="8" width="21.33203125" style="21" customWidth="1"/>
+    <col min="9" max="16381" width="11.5546875" style="13"/>
+    <col min="16382" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:8">
       <c r="A1" s="15" t="s">
         <v>116</v>
       </c>
@@ -1753,21 +1749,18 @@
         <v>106</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="H1" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="H1" s="21" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1784,23 +1777,22 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE5D49AE-AF0F-4668-A81E-764A0CB4B708}">
-  <dimension ref="A1:XFB1"/>
+  <dimension ref="A1:XFA1"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="28.109375" style="13" customWidth="1"/>
     <col min="2" max="2" width="24.33203125" style="20" customWidth="1"/>
     <col min="3" max="3" width="36.88671875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="13" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" style="13" customWidth="1"/>
-    <col min="7" max="7" width="24.6640625" style="13" customWidth="1"/>
-    <col min="8" max="8" width="17" style="13" customWidth="1"/>
-    <col min="9" max="9" width="21.6640625" style="21" customWidth="1"/>
-    <col min="10" max="16382" width="11.5546875" style="13"/>
-    <col min="16383" max="16384" width="11.5546875" style="14"/>
+    <col min="4" max="4" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" style="13" customWidth="1"/>
+    <col min="6" max="6" width="24.6640625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="17" style="13" customWidth="1"/>
+    <col min="8" max="8" width="21.6640625" style="21" customWidth="1"/>
+    <col min="9" max="16381" width="11.5546875" style="13"/>
+    <col min="16382" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:8">
       <c r="A1" s="15" t="s">
         <v>116</v>
       </c>
@@ -1811,21 +1803,18 @@
         <v>106</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="H1" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="H1" s="21" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1841,23 +1830,23 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:XFC6"/>
+  <dimension ref="A1:XFB6"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="13" customWidth="1"/>
     <col min="2" max="2" width="16.88671875" style="20" customWidth="1"/>
-    <col min="3" max="4" width="18.88671875" style="13" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="17.33203125" style="13" customWidth="1"/>
-    <col min="8" max="8" width="20.6640625" style="21" customWidth="1"/>
-    <col min="9" max="9" width="22.44140625" style="13" customWidth="1"/>
-    <col min="10" max="10" width="24" style="13" customWidth="1"/>
-    <col min="11" max="12" width="22.33203125" style="13" customWidth="1"/>
-    <col min="14" max="16383" width="11.5546875" style="13"/>
-    <col min="16384" max="16384" width="11.5546875" style="14"/>
+    <col min="3" max="3" width="18.88671875" style="13" customWidth="1"/>
+    <col min="4" max="4" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17.33203125" style="13" customWidth="1"/>
+    <col min="7" max="7" width="20.6640625" style="21" customWidth="1"/>
+    <col min="8" max="8" width="22.44140625" style="13" customWidth="1"/>
+    <col min="9" max="9" width="24" style="13" customWidth="1"/>
+    <col min="10" max="11" width="22.33203125" style="13" customWidth="1"/>
+    <col min="13" max="16382" width="11.5546875" style="13"/>
+    <col min="16383" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:11">
       <c r="A1" s="15" t="s">
         <v>116</v>
       </c>
@@ -1868,43 +1857,39 @@
         <v>106</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="G1" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="G1" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="H1" s="15" t="s">
         <v>109</v>
       </c>
+      <c r="I1" s="13" t="s">
+        <v>110</v>
+      </c>
       <c r="J1" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="L1" s="13" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:11">
       <c r="A6" s="15"/>
       <c r="B6" s="19"/>
       <c r="C6" s="15"/>
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>

</xml_diff>

<commit_message>
v0.20.33 with si6 folder
</commit_message>
<xml_diff>
--- a/auto_repair/public/www/assets/xlsx/si-6.xlsx
+++ b/auto_repair/public/www/assets/xlsx/si-6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abees\Documents\sic\auto-repair-erp\web\src\assets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15BFA07-2AFD-45E6-BDDD-2C1A998743FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656B2AB4-843D-46E1-91CF-15469E79002C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fiscal Years" sheetId="1" r:id="rId1"/>
@@ -32,9 +32,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Journal Entries'!$A$1:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Products!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Raw Material'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Trading!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Products!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Raw Material'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Trading!$A$1:$H$1</definedName>
     <definedName name="arial" localSheetId="13">Invoices!$1:$1048576</definedName>
     <definedName name="arial">#REF!</definedName>
   </definedNames>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="125">
   <si>
     <t>year</t>
   </si>
@@ -429,6 +429,9 @@
   </si>
   <si>
     <t>system</t>
+  </si>
+  <si>
+    <t>Is Recycable</t>
   </si>
 </sst>
 </file>
@@ -1723,22 +1726,23 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD83FC68-3866-4B53-B82D-AC812A1EEF62}">
-  <dimension ref="A1:XFA1"/>
+  <dimension ref="A1:XFB1"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="13" customWidth="1"/>
     <col min="2" max="2" width="24.33203125" style="20" customWidth="1"/>
     <col min="3" max="3" width="36.88671875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" style="13" customWidth="1"/>
-    <col min="6" max="6" width="24.6640625" style="13" customWidth="1"/>
-    <col min="7" max="7" width="17" style="13" customWidth="1"/>
-    <col min="8" max="8" width="21.33203125" style="21" customWidth="1"/>
-    <col min="9" max="16381" width="11.5546875" style="13"/>
-    <col min="16382" max="16384" width="11.5546875" style="14"/>
+    <col min="4" max="4" width="17.6640625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="24.6640625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="17" style="13" customWidth="1"/>
+    <col min="9" max="9" width="21.33203125" style="21" customWidth="1"/>
+    <col min="10" max="16382" width="11.5546875" style="13"/>
+    <col min="16383" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="15" t="s">
         <v>116</v>
       </c>
@@ -1749,18 +1753,21 @@
         <v>106</v>
       </c>
       <c r="D1" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="H1" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="I1" s="21" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1777,22 +1784,23 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE5D49AE-AF0F-4668-A81E-764A0CB4B708}">
-  <dimension ref="A1:XFA1"/>
+  <dimension ref="A1:XFB1"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="28.109375" style="13" customWidth="1"/>
     <col min="2" max="2" width="24.33203125" style="20" customWidth="1"/>
     <col min="3" max="3" width="36.88671875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" style="13" customWidth="1"/>
-    <col min="6" max="6" width="24.6640625" style="13" customWidth="1"/>
-    <col min="7" max="7" width="17" style="13" customWidth="1"/>
-    <col min="8" max="8" width="21.6640625" style="21" customWidth="1"/>
-    <col min="9" max="16381" width="11.5546875" style="13"/>
-    <col min="16382" max="16384" width="11.5546875" style="14"/>
+    <col min="4" max="4" width="15.33203125" style="13" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="24.6640625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="17" style="13" customWidth="1"/>
+    <col min="9" max="9" width="21.6640625" style="21" customWidth="1"/>
+    <col min="10" max="16382" width="11.5546875" style="13"/>
+    <col min="16383" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="15" t="s">
         <v>116</v>
       </c>
@@ -1803,18 +1811,21 @@
         <v>106</v>
       </c>
       <c r="D1" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="H1" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="I1" s="21" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1830,23 +1841,23 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:XFB6"/>
+  <dimension ref="A1:XFC6"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="13" customWidth="1"/>
     <col min="2" max="2" width="16.88671875" style="20" customWidth="1"/>
-    <col min="3" max="3" width="18.88671875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="17.33203125" style="13" customWidth="1"/>
-    <col min="7" max="7" width="20.6640625" style="21" customWidth="1"/>
-    <col min="8" max="8" width="22.44140625" style="13" customWidth="1"/>
-    <col min="9" max="9" width="24" style="13" customWidth="1"/>
-    <col min="10" max="11" width="22.33203125" style="13" customWidth="1"/>
-    <col min="13" max="16382" width="11.5546875" style="13"/>
-    <col min="16383" max="16384" width="11.5546875" style="14"/>
+    <col min="3" max="4" width="18.88671875" style="13" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.33203125" style="13" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" style="21" customWidth="1"/>
+    <col min="9" max="9" width="22.44140625" style="13" customWidth="1"/>
+    <col min="10" max="10" width="24" style="13" customWidth="1"/>
+    <col min="11" max="12" width="22.33203125" style="13" customWidth="1"/>
+    <col min="14" max="16383" width="11.5546875" style="13"/>
+    <col min="16384" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="15" t="s">
         <v>116</v>
       </c>
@@ -1857,39 +1868,43 @@
         <v>106</v>
       </c>
       <c r="D1" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="H1" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="I1" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" s="15"/>
       <c r="B6" s="19"/>
       <c r="C6" s="15"/>
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="G6" s="15"/>
       <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>

</xml_diff>